<commit_message>
refactor: improve data handling in logit table generation by refining dropna logic for CNN-only models; update Excel outputs for consistency across US and CN tables
</commit_message>
<xml_diff>
--- a/outputs/05_benchmark_signals/tables_v_viii/cn/table_vii_return_logit.xlsx
+++ b/outputs/05_benchmark_signals/tables_v_viii/cn/table_vii_return_logit.xlsx
@@ -473,7 +473,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>3.85*** (6.8)</t>
+          <t>1.60*** (3.0)</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
@@ -484,7 +484,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2.45*** (5.1)</t>
+          <t>0.77*** (3.7)</t>
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
@@ -495,7 +495,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>1.85*** (4.8)</t>
+          <t>0.48*** (3.5)</t>
         </is>
       </c>
       <c r="I2" t="inlineStr"/>
@@ -1070,7 +1070,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>3.85***</t>
+          <t>1.60***</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
@@ -1081,7 +1081,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2.45***</t>
+          <t>0.77***</t>
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
@@ -1092,7 +1092,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>1.85***</t>
+          <t>0.48***</t>
         </is>
       </c>
       <c r="I2" t="inlineStr"/>
@@ -1711,42 +1711,42 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>3.853854232918517</v>
+        <v>1.596704469189518</v>
       </c>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="n">
         <v>1.011287241894017</v>
       </c>
       <c r="E2" t="n">
-        <v>2.446774616065345</v>
+        <v>0.773573037475353</v>
       </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="n">
         <v>0.1593852846071442</v>
       </c>
       <c r="H2" t="n">
-        <v>1.852542399227079</v>
+        <v>0.4833046761211478</v>
       </c>
       <c r="I2" t="inlineStr"/>
       <c r="J2" t="n">
         <v>0.07453220317442487</v>
       </c>
       <c r="K2" t="n">
-        <v>6.834812349752647</v>
+        <v>3.02526678272412</v>
       </c>
       <c r="L2" t="inlineStr"/>
       <c r="M2" t="n">
         <v>2.378269714906367</v>
       </c>
       <c r="N2" t="n">
-        <v>5.077304916846577</v>
+        <v>3.745987916569298</v>
       </c>
       <c r="O2" t="inlineStr"/>
       <c r="P2" t="n">
         <v>1.259523968718567</v>
       </c>
       <c r="Q2" t="n">
-        <v>4.757403846245063</v>
+        <v>3.497027205059362</v>
       </c>
       <c r="R2" t="inlineStr"/>
       <c r="S2" t="n">

</xml_diff>